<commit_message>
Merged PR 3054: Merge DeepikaRefactoringGrey to master-grey
</commit_message>
<xml_diff>
--- a/src/main/resources/Negotiations_Field_Values.xlsx
+++ b/src/main/resources/Negotiations_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7406A7-090D-4A8C-B410-04AC660316E8}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D4A5CA-5F6D-4D0A-99D1-058BCA43344C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
@@ -53,13 +53,13 @@
     <t>Negoatiation Initiated</t>
   </si>
   <si>
-    <t>Budget: Focus Area</t>
-  </si>
-  <si>
     <t>Attachments: Notes</t>
   </si>
   <si>
     <t>Budget: Budget Details</t>
+  </si>
+  <si>
+    <t>Overview: Project Information</t>
   </si>
 </sst>
 </file>
@@ -380,7 +380,7 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.5546875" customWidth="1"/>
     <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -414,7 +414,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -474,7 +474,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -533,7 +533,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
made changes in user and url
</commit_message>
<xml_diff>
--- a/src/main/resources/Negotiations_Field_Values.xlsx
+++ b/src/main/resources/Negotiations_Field_Values.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A9D039-8841-4FA7-A1A7-DFAF934692A6}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B7E6C43-7C1D-4F03-9B3D-4D8A59F74D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
-    <sheet name="App Revision" sheetId="4" r:id="rId2"/>
-    <sheet name="Due Date" sheetId="5" r:id="rId3"/>
-    <sheet name="Edition1" sheetId="2" r:id="rId4"/>
-    <sheet name="Edition2" sheetId="3" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId2"/>
+    <sheet name="App Revision" sheetId="4" r:id="rId3"/>
+    <sheet name="Due Date" sheetId="5" r:id="rId4"/>
+    <sheet name="Edition1" sheetId="2" r:id="rId5"/>
+    <sheet name="Edition2" sheetId="3" r:id="rId6"/>
+    <sheet name="Edition_Forms" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="15">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -62,19 +64,37 @@
   </si>
   <si>
     <t>Overview: Project Information</t>
+  </si>
+  <si>
+    <t>fieldApplicationSectionsForRevision__c</t>
+  </si>
+  <si>
+    <t>fieldTEXTAREAExplanationOfRevisionsNeeded__c</t>
+  </si>
+  <si>
+    <t>fieldNegotiationDueDate__c</t>
+  </si>
+  <si>
+    <t>Files: Forms</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF202124"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -97,8 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,13 +401,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="48.53125" customWidth="1"/>
-    <col min="3" max="3" width="25.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.5703125" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -397,34 +418,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>4</v>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="C4">
         <v>43707</v>
@@ -437,15 +458,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E662A116-3984-4CDE-8E67-B1843A9454D2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA7FEAA1-1569-4FC1-85CC-6DA4026B11F4}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="48.53125" customWidth="1"/>
-    <col min="3" max="3" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -456,7 +486,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -467,7 +497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -483,16 +513,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C06C4F7E-796A-4AC4-AC16-D1680880C5DA}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="48.53125" customWidth="1"/>
-    <col min="3" max="3" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -503,7 +533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -514,7 +544,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -530,17 +560,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E8A2259-147F-4561-A3B1-EDF044621ED4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -551,7 +581,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -562,7 +592,7 @@
         <v>43707</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -573,7 +603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -589,17 +619,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E8146D-F630-4D59-97ED-A466989510BA}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -610,7 +640,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -621,7 +651,7 @@
         <v>43707</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -632,7 +662,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -641,6 +671,65 @@
       </c>
       <c r="C4" t="s">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FE65BFC-6AFF-4E04-B5FE-B40621538AA3}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4">
+        <v>43707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>